<commit_message>
Update backoffice and exclude source archive
</commit_message>
<xml_diff>
--- a/testing_files/test8 - pubmed upload hcp file/Sample HCPs Italy.xlsx
+++ b/testing_files/test8 - pubmed upload hcp file/Sample HCPs Italy.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TomásCarrilho\GitHub-Projects\gds-backoffice\testing_files\test8 - pubmed upload hcp file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6F55B5F-2FDC-4D11-9C00-6F869610F82E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5616CDC8-E84C-471B-9B82-2C92E5A76381}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2910" windowWidth="29040" windowHeight="15720" xr2:uid="{B4DDF21F-2EED-4ED8-96C9-35D8674993D3}"/>
+    <workbookView xWindow="10" yWindow="10" windowWidth="25580" windowHeight="15260" activeTab="1" xr2:uid="{B4DDF21F-2EED-4ED8-96C9-35D8674993D3}"/>
   </bookViews>
   <sheets>
     <sheet name="sample" sheetId="1" r:id="rId1"/>
+    <sheet name="second" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1142,4 +1143,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2251306-055D-4F26-A57D-39F949E8EFA3}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>